<commit_message>
update de : in rcnv excel
</commit_message>
<xml_diff>
--- a/resources/rCNV/docs/recurrent_CNV_dataset.xlsx
+++ b/resources/rCNV/docs/recurrent_CNV_dataset.xlsx
@@ -622,7 +622,7 @@
     <t xml:space="preserve">15q24 recurrent region (LCR C-LCR D) (includes SIN3A)</t>
   </si>
   <si>
-    <t xml:space="preserve">15: 75631787-75972909</t>
+    <t xml:space="preserve">15:75631787-75972909</t>
   </si>
   <si>
     <t xml:space="preserve">15:75339446-75680568</t>
@@ -1296,7 +1296,7 @@
     <t xml:space="preserve">X:48306152-52103258</t>
   </si>
   <si>
-    <t xml:space="preserve">X: 48447780-52444264</t>
+    <t xml:space="preserve">X:48447780-52444264</t>
   </si>
   <si>
     <t xml:space="preserve">12/14/2017</t>

</xml_diff>